<commit_message>
Updated the sample synthetic data with fewer files
</commit_message>
<xml_diff>
--- a/data_raw/samples/exchange_rates.xlsx
+++ b/data_raw/samples/exchange_rates.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="18">
   <si>
     <t>date</t>
   </si>
@@ -25,22 +25,49 @@
     <t>rate_to_aud</t>
   </si>
   <si>
+    <t>2025-10-12</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>GBP</t>
+  </si>
+  <si>
+    <t>JPY</t>
+  </si>
+  <si>
+    <t>2025-10-13</t>
+  </si>
+  <si>
+    <t>2025-10-14</t>
+  </si>
+  <si>
+    <t>2025-10-15</t>
+  </si>
+  <si>
+    <t>2025-10-16</t>
+  </si>
+  <si>
+    <t>2025-10-17</t>
+  </si>
+  <si>
+    <t>2025-10-18</t>
+  </si>
+  <si>
+    <t>2025-10-19</t>
+  </si>
+  <si>
     <t>2025-10-20</t>
   </si>
   <si>
-    <t>USD</t>
-  </si>
-  <si>
-    <t>EUR</t>
-  </si>
-  <si>
-    <t>GBP</t>
-  </si>
-  <si>
-    <t>JPY</t>
-  </si>
-  <si>
     <t>2025-10-21</t>
+  </si>
+  <si>
+    <t>2025-10-22</t>
   </si>
 </sst>
 </file>
@@ -372,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -394,7 +421,7 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>0.6963204200000001</v>
+        <v>0.69718357</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -405,7 +432,7 @@
         <v>5</v>
       </c>
       <c r="C3">
-        <v>0.65207459</v>
+        <v>0.65330868</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -416,7 +443,7 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>0.48631539</v>
+        <v>0.49293844</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -427,7 +454,7 @@
         <v>7</v>
       </c>
       <c r="C5">
-        <v>97.91305838</v>
+        <v>97.91761515</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -438,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>0.70147542</v>
+        <v>0.6960128</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -449,7 +476,7 @@
         <v>5</v>
       </c>
       <c r="C7">
-        <v>0.65673099</v>
+        <v>0.652138</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -460,7 +487,7 @@
         <v>6</v>
       </c>
       <c r="C8">
-        <v>0.4821193</v>
+        <v>0.5008345</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -471,7 +498,403 @@
         <v>7</v>
       </c>
       <c r="C9">
-        <v>97.91151232</v>
+        <v>97.92145232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10">
+        <v>0.69366543</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11">
+        <v>0.6548508</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12">
+        <v>0.49851741</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13">
+        <v>97.91912367</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14">
+        <v>0.69487524</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15">
+        <v>0.6452844</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16">
+        <v>0.48989282</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17">
+        <v>97.91631223</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>0.68981108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19">
+        <v>0.64685564</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20">
+        <v>0.4853527</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21">
+        <v>97.90925070999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22">
+        <v>0.69713932</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23">
+        <v>0.64572676</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24">
+        <v>0.48569034</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25">
+        <v>97.90212697</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26">
+        <v>0.69441741</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27">
+        <v>0.64628137</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28">
+        <v>0.47993537</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>13</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29">
+        <v>97.90400545999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30">
+        <v>0.69141422</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31">
+        <v>0.6448229</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>14</v>
+      </c>
+      <c r="B32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32">
+        <v>0.47692684</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33">
+        <v>97.91326685</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34">
+        <v>0.69134673</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>15</v>
+      </c>
+      <c r="B35" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35">
+        <v>0.63953435</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36">
+        <v>0.48103956</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37">
+        <v>97.90716263</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>16</v>
+      </c>
+      <c r="B38" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38">
+        <v>0.69239105</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39">
+        <v>0.629736</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>16</v>
+      </c>
+      <c r="B40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40">
+        <v>0.47439863</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41">
+        <v>97.90814693999999</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42">
+        <v>0.69608338</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43">
+        <v>0.63059284</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B44" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44">
+        <v>0.47382039</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45">
+        <v>97.90664142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>